<commit_message>
fix fluo, C_org and UV names
</commit_message>
<xml_diff>
--- a/Initial data/2025/TOC.xlsx
+++ b/Initial data/2025/TOC.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="126">
   <si>
-    <t>Sample</t>
+    <t>Sample Name</t>
   </si>
   <si>
     <t>C_org</t>
@@ -41,58 +41,58 @@
     <t>CV Conc</t>
   </si>
   <si>
-    <t>ADOM-SLB-1</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-L1</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-L2</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-L3</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-S</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-M1</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-M2</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-1-M3</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2-1-marker</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2-1-pen</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2-2</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2-K-1</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-2-luzha</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-3-1</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-3-2</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-3-3</t>
-  </si>
-  <si>
-    <t>ADOM-SLB-Z1-M</t>
+    <t>ADOM-SLB-B-1</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-6</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-7</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-8</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-5</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-1</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-2</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-3</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B-2</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B-2-1-marker</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B-2-1-pen</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B2-2</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B2-3</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B1-4</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B3-1</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B3-2</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-B3-3</t>
+  </si>
+  <si>
+    <t>ADOM-SLB-BZ-1</t>
   </si>
   <si>
     <t>ADOM-SLB-BO-1</t>
@@ -1402,7 +1402,7 @@
   <dimension ref="A1:D136"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="1" max="1" width="32.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">

</xml_diff>